<commit_message>
added expense analysis and chart files
</commit_message>
<xml_diff>
--- a/expense_report.xlsx
+++ b/expense_report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -431,51 +431,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Bills</t>
+          <t>Food</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3700</v>
+        <v>500</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Entertainment</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1100</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Food</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1750</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
           <t>Shopping</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Travel</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>450</v>
+      <c r="B4" t="n">
+        <v>1200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated expense analysis project
</commit_message>
<xml_diff>
--- a/expense_report.xlsx
+++ b/expense_report.xlsx
@@ -413,49 +413,229 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Amount</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Description</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Food</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="C2" t="n">
         <v>500</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Travel</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>200</v>
+      <c r="C3" t="n">
+        <v>300</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Bus Ticket</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>Shopping</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="C4" t="n">
         <v>1200</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Clothes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-01-08</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bills</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>800</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Electricity Bill</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>600</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Movie</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Doctor Visit</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>450</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>700</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Train Ticket</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Shopping</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>900</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Shoes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Bills</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Internet Bill</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>